<commit_message>
Palazzo Simonetti: luogo trasformato, ancorato a via Lanza (T-11, D-032)
Palazzo reale di via Lata che Gadda colloca in via Lanza: Transformed,
senza coordinate proprie. L'entità del gazetteer di via Vittoria Colonna
diventa gaz_palazzo_odescalchi_simonetti (lettura di Terzoli).
ABox 16.055 -> 16.057, full 17.225 -> 17.227, SHACL conforme. Chiude DC-02.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/GazetteerEntities.xlsx
+++ b/data/source/xlsx/GazetteerEntities.xlsx
@@ -5071,12 +5071,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>gaz_palazzo_simonetti</t>
+          <t>gaz_palazzo_odescalchi_simonetti</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Palazzo Simonetti</t>
+          <t>Palazzo Odescalchi Simonetti</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -5112,6 +5112,11 @@
     }
   ]
 }</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Candidato della lettura di Terzoli (cit. in Pinotti 2025, p. 78): palazzo Odescalchi Simonetti, già pensione White, dove Gadda aveva abitato. Civico 11 secondo Pinotti; il dato precedente indicava 13. Non è il referente di palazzo_simonetti: entità predisposta per l'identificazione attribuita.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 3d, B1: statuti dei casi vicini secondo Terzoli 2015; note del censimento (D-092)
Castel Porcano Transformed (S-castel_porcano-3, I-0012, N-0007); via delle Oche
Imported, a Milano (gaz_via_delle_oche_milano, S-via_delle_oche-2, I-0013,
interp_00979, U-0009 non adottata); pensione Burgess Invented con motivazione
nuova e ancora gaz_roma (S-pensione_burgess-2, interp_00980-00982); Rocca Orsina
identificata (I-0014); Monte Nuncupale: ipotesi di Terzoli non adottata (I-0015,
gaz_campidoglio). Note di due_santi, marino, monte_manno svuotate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/GazetteerEntities.xlsx
+++ b/data/source/xlsx/GazetteerEntities.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K270"/>
+  <dimension ref="A1:K272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6947,6 +6947,11 @@
 }</t>
         </is>
       </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Terzoli 2015, pp. 507–508 (identificazione); coordinata nell'area di Palazzo Colonna, che occupa il sedime della rocca; coordinata verificata sul poligono OSM di Palazzo Colonna, way 74413768.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -12658,6 +12663,85 @@
       <c r="J270" t="inlineStr">
         <is>
           <t>Bertarelli 1925, cart. 4, secondo Terzoli 2015, pp. 418–419, 911. Senza coordinate; il luogo ponte_di_santa_fumia resta ancorato a gaz_quarto_di_santa_fumia (D-087).</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>gaz_via_delle_oche_milano</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>via delle Oche</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Via di Okk</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>contrada milanese scomparsa</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>via Bernardino Zenale, Milano, tra via San Vittore e corso Magenta, presso Santa Maria delle Grazie</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>45.464649</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>9.170031</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>{
+  "type": "FeatureCollection",
+  "features": [
+    {
+      "type": "Feature",
+      "properties": {},
+      "geometry": {
+        "type": "Point",
+        "coordinates": [
+          9.170031,
+          45.464649
+        ]
+      }
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Terzoli 2015, p. 77; L'Adalgisa, p. 564, n. 53. Coordinata: centroide di via Bernardino Zenale, OpenStreetMap, way 27756097 e 286239491.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>gaz_campidoglio</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Campidoglio</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Senza coordinate: bersaglio dell'identificazione non adottata I-0015 (Terzoli 2015, pp. 507–508).</t>
         </is>
       </c>
     </row>

</xml_diff>